<commit_message>
updating capps model to ne variant and cleaning plotting_comparisons script
</commit_message>
<xml_diff>
--- a/analyses/figures/zarchive/harvests_approaches.xlsx
+++ b/analyses/figures/zarchive/harvests_approaches.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/CatherineChamberlain/Documents/git/dynamic_carbonaccounting/analyses/figures/zarchive/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/c.chamberlain/Documents/git/dynamic_carbonaccounting/analyses/figures/zarchive/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15FCB73-A0E0-6B4C-999E-FB627D523117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF83787A-954C-4C47-B1A4-44B031E7680A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="15600" xr2:uid="{674C4B86-B71C-9F45-B66A-38E4338ED408}"/>
+    <workbookView xWindow="660" yWindow="660" windowWidth="28040" windowHeight="15600" activeTab="1" xr2:uid="{674C4B86-B71C-9F45-B66A-38E4338ED408}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -613,6 +613,12 @@
       <c r="E3" s="8">
         <v>0.34410000000000002</v>
       </c>
+      <c r="F3" s="8">
+        <v>0.12</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -652,6 +658,12 @@
       </c>
       <c r="E5" s="8">
         <v>0.34410000000000002</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0.32</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0.27</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -922,6 +934,12 @@
       <c r="E3" s="8">
         <v>0.33510000000000001</v>
       </c>
+      <c r="F3" s="8">
+        <v>0.18</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0.26</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -961,6 +979,12 @@
       </c>
       <c r="E5" s="8">
         <v>0.33510000000000001</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0.48</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0.3</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>